<commit_message>
add new regional trade scenario figures
</commit_message>
<xml_diff>
--- a/Inputs/Dict/Dict_Scenario.xlsx
+++ b/Inputs/Dict/Dict_Scenario.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Pablo\Educacion\Aprendizaje Continuo\Codigos utiles\R\Proyectos R\EV-Minerals-MONET\Inputs\Dict\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Pablo\Educacion\Programming\R\R UC Davis\ETM-Regional-Sufficiency-Circularity\Inputs\Dict\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{573484AE-F131-4354-B8D4-F936DA7D7253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C781EE4E-26E3-4E76-83C2-6780E84BCDEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{49FC0923-77E1-4464-87AC-6180D1E2433D}"/>
+    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{49FC0923-77E1-4464-87AC-6180D1E2433D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="51">
   <si>
     <t>name</t>
   </si>
@@ -183,6 +183,12 @@
   </si>
   <si>
     <t>China expansion</t>
+  </si>
+  <si>
+    <t>MONET_RegionalHighDS</t>
+  </si>
+  <si>
+    <t>Regional Higher Domestic Supply</t>
   </si>
 </sst>
 </file>
@@ -563,7 +569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCAAB542-BAC6-4E48-AB9F-79F031AAB640}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
@@ -742,24 +748,24 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -770,10 +776,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -784,10 +790,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -798,21 +804,24 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B18" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -820,10 +829,10 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -831,35 +840,32 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B20" t="s">
         <v>8</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B21" t="s">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="C21">
         <v>1</v>
-      </c>
-      <c r="D21" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -870,15 +876,29 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>43</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>45</v>
       </c>
-      <c r="C23">
-        <v>1</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24" t="s">
         <v>44</v>
       </c>
     </row>

</xml_diff>